<commit_message>
Pennylane : alignement sur l'OpenAPI officielle de POST /billing_subscriptions
- mapping et client : mode {type}, payment_conditions, payment_method,
  recurring_rule (monthly interval 1/3/6, yearly), customer_invoice_data
  (currency, language, pdf_invoice_subject, special_mention d'indexation,
  invoice_lines avec unit et raw_currency_unit_price en chaîne)
- réglages communs (mode, conditions, moyen de paiement) dans la feuille
  Société avec listes déroulantes ; colonne « Pennylane subscription_id »
  dans Baux, remplie après un 201, refus de doublon sauf --remplacer
- feuille Pennylane régénérée : le JSON par formules est comparé au corps
  du client Python dans le test de parité LibreOffice
- INSEE : option --api-insee (api.insee.fr/series/BDM, jeton INSEE_API_TOKEN)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBWZYnWmN9TckE8aBoYJon
</commit_message>
<xml_diff>
--- a/demo/DEMO_SCI_EXEMPLE_valeurs_fictives.xlsx
+++ b/demo/DEMO_SCI_EXEMPLE_valeurs_fictives.xlsx
@@ -114,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,9 +144,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -912,7 +909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1039,26 +1036,73 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Date de génération</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="n">
-        <v>46274</v>
+          <t>Pennylane – mode des factures</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>awaiting_validation</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
+          <t>Pennylane – conditions de paiement</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>upon_receipt</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Pennylane – moyen de paiement</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>offline</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Date de génération</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>46274</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
           <t>Mode démonstration</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>OUI</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"awaiting_validation,finalized"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"upon_receipt,7_days,15_days,30_days,30_days_end_of_month,45_days,45_days_end_of_month,60_days"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"offline,gocardless_direct_debit,pro_account_sepa_core"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1069,7 +1113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1091,8 +1135,9 @@
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="30" customWidth="1" min="20" max="20"/>
-    <col width="40" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -1193,10 +1238,15 @@
       </c>
       <c r="T1" s="10" t="inlineStr">
         <is>
+          <t>Pennylane subscription_id</t>
+        </is>
+      </c>
+      <c r="U1" s="10" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="U1" s="10" t="inlineStr">
+      <c r="V1" s="10" t="inlineStr">
         <is>
           <t>Contrôles</t>
         </is>
@@ -1278,12 +1328,13 @@
         </is>
       </c>
       <c r="S2" s="11" t="n"/>
-      <c r="T2" s="11" t="inlineStr">
+      <c r="T2" s="11" t="n"/>
+      <c r="U2" s="11" t="inlineStr">
         <is>
           <t>Clause d'échelle mobile annuelle, ILC même trimestre</t>
         </is>
       </c>
-      <c r="U2" s="15">
+      <c r="V2" s="15">
         <f>IF(A2="","",TRIM(IF(F2="","Date d'effet manquante. ","")&amp;IF(NOT(ISNUMBER(I2)),"Loyer initial manquant. ","")&amp;IF(COUNTIF(Indices!$A:$A,M2)=0,"Aucune valeur d'indice chargée pour cette série. ","")&amp;IF(SUMIFS(Indices!$C:$C,Indices!$A:$A,M2,Indices!$B:$B,N2)=0,"Indice de base "&amp;N2&amp;" absent de la feuille Indices. ","")&amp;IF(LEN(N2)&lt;&gt;7,"Trimestre de base au format AAAA-Tn. ","")&amp;IF(COUNTIF($A$2:$A$200,A2)&gt;1,"ID bail en doublon. ","")&amp;IF(AND(Q2&lt;&gt;"",NOT(ISNUMBER(Q2))),"Plafond non numérique. ","")&amp;IF(COUNTIF($A$2:$A$200,A2)=1,"",""))&amp;IF(AND(F2&lt;&gt;"",ISNUMBER(I2),SUMIFS(Indices!$C:$C,Indices!$A:$A,M2,Indices!$B:$B,N2)&gt;0,LEN(N2)=7,COUNTIF($A$2:$A$200,A2)=1),"OK",""))</f>
         <v/>
       </c>
@@ -1359,12 +1410,13 @@
         </is>
       </c>
       <c r="S3" s="11" t="n"/>
-      <c r="T3" s="11" t="inlineStr">
+      <c r="T3" s="11" t="n"/>
+      <c r="U3" s="11" t="inlineStr">
         <is>
           <t>Révision triennale indexée ILAT, indice de base fixe</t>
         </is>
       </c>
-      <c r="U3" s="15">
+      <c r="V3" s="15">
         <f>IF(A3="","",TRIM(IF(F3="","Date d'effet manquante. ","")&amp;IF(NOT(ISNUMBER(I3)),"Loyer initial manquant. ","")&amp;IF(COUNTIF(Indices!$A:$A,M3)=0,"Aucune valeur d'indice chargée pour cette série. ","")&amp;IF(SUMIFS(Indices!$C:$C,Indices!$A:$A,M3,Indices!$B:$B,N3)=0,"Indice de base "&amp;N3&amp;" absent de la feuille Indices. ","")&amp;IF(LEN(N3)&lt;&gt;7,"Trimestre de base au format AAAA-Tn. ","")&amp;IF(COUNTIF($A$2:$A$200,A3)&gt;1,"ID bail en doublon. ","")&amp;IF(AND(Q3&lt;&gt;"",NOT(ISNUMBER(Q3))),"Plafond non numérique. ","")&amp;IF(COUNTIF($A$2:$A$200,A3)=1,"",""))&amp;IF(AND(F3&lt;&gt;"",ISNUMBER(I3),SUMIFS(Indices!$C:$C,Indices!$A:$A,M3,Indices!$B:$B,N3)&gt;0,LEN(N3)=7,COUNTIF($A$2:$A$200,A3)=1),"OK",""))</f>
         <v/>
       </c>
@@ -1438,12 +1490,13 @@
       </c>
       <c r="R4" s="11" t="n"/>
       <c r="S4" s="11" t="n"/>
-      <c r="T4" s="11" t="inlineStr">
+      <c r="T4" s="11" t="n"/>
+      <c r="U4" s="11" t="inlineStr">
         <is>
           <t>Bail antérieur à 2014 renouvelé, clause ICC ; plafond contractuel 3,5 %</t>
         </is>
       </c>
-      <c r="U4" s="15">
+      <c r="V4" s="15">
         <f>IF(A4="","",TRIM(IF(F4="","Date d'effet manquante. ","")&amp;IF(NOT(ISNUMBER(I4)),"Loyer initial manquant. ","")&amp;IF(COUNTIF(Indices!$A:$A,M4)=0,"Aucune valeur d'indice chargée pour cette série. ","")&amp;IF(SUMIFS(Indices!$C:$C,Indices!$A:$A,M4,Indices!$B:$B,N4)=0,"Indice de base "&amp;N4&amp;" absent de la feuille Indices. ","")&amp;IF(LEN(N4)&lt;&gt;7,"Trimestre de base au format AAAA-Tn. ","")&amp;IF(COUNTIF($A$2:$A$200,A4)&gt;1,"ID bail en doublon. ","")&amp;IF(AND(Q4&lt;&gt;"",NOT(ISNUMBER(Q4))),"Plafond non numérique. ","")&amp;IF(COUNTIF($A$2:$A$200,A4)=1,"",""))&amp;IF(AND(F4&lt;&gt;"",ISNUMBER(I4),SUMIFS(Indices!$C:$C,Indices!$A:$A,M4,Indices!$B:$B,N4)&gt;0,LEN(N4)=7,COUNTIF($A$2:$A$200,A4)=1),"OK",""))</f>
         <v/>
       </c>
@@ -1515,20 +1568,21 @@
       <c r="Q5" s="11" t="n"/>
       <c r="R5" s="11" t="n"/>
       <c r="S5" s="11" t="n"/>
-      <c r="T5" s="11" t="inlineStr">
+      <c r="T5" s="11" t="n"/>
+      <c r="U5" s="11" t="inlineStr">
         <is>
           <t>customer_id Pennylane à créer</t>
         </is>
       </c>
-      <c r="U5" s="15">
+      <c r="V5" s="15">
         <f>IF(A5="","",TRIM(IF(F5="","Date d'effet manquante. ","")&amp;IF(NOT(ISNUMBER(I5)),"Loyer initial manquant. ","")&amp;IF(COUNTIF(Indices!$A:$A,M5)=0,"Aucune valeur d'indice chargée pour cette série. ","")&amp;IF(SUMIFS(Indices!$C:$C,Indices!$A:$A,M5,Indices!$B:$B,N5)=0,"Indice de base "&amp;N5&amp;" absent de la feuille Indices. ","")&amp;IF(LEN(N5)&lt;&gt;7,"Trimestre de base au format AAAA-Tn. ","")&amp;IF(COUNTIF($A$2:$A$200,A5)&gt;1,"ID bail en doublon. ","")&amp;IF(AND(Q5&lt;&gt;"",NOT(ISNUMBER(Q5))),"Plafond non numérique. ","")&amp;IF(COUNTIF($A$2:$A$200,A5)=1,"",""))&amp;IF(AND(F5&lt;&gt;"",ISNUMBER(I5),SUMIFS(Indices!$C:$C,Indices!$A:$A,M5,Indices!$B:$B,N5)&gt;0,LEN(N5)=7,COUNTIF($A$2:$A$200,A5)=1),"OK",""))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="U2:U200">
+  <conditionalFormatting sqref="V2:V200">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND(U2&lt;&gt;"",U2&lt;&gt;"OK")</formula>
+      <formula>AND(V2&lt;&gt;"",V2&lt;&gt;"OK")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -10415,22 +10469,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="90" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="100" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -10456,7 +10516,7 @@
       </c>
       <c r="E1" s="10" t="inlineStr">
         <is>
-          <t>Libellé de ligne</t>
+          <t>label (abonnement)</t>
         </is>
       </c>
       <c r="F1" s="10" t="inlineStr">
@@ -10466,37 +10526,67 @@
       </c>
       <c r="G1" s="10" t="inlineStr">
         <is>
-          <t>recurrence.type</t>
+          <t>recurring_rule.type</t>
         </is>
       </c>
       <c r="H1" s="10" t="inlineStr">
         <is>
+          <t>interval</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
           <t>Prix unitaire HT / échéance</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="K1" s="10" t="inlineStr">
         <is>
           <t>Charges HT / échéance</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="L1" s="10" t="inlineStr">
         <is>
           <t>TVA (%)</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
-        <is>
-          <t>vat_rate (code Pennylane)</t>
-        </is>
-      </c>
-      <c r="L1" s="10" t="inlineStr">
-        <is>
-          <t>Date de début (1er du mois suivant)</t>
-        </is>
-      </c>
       <c r="M1" s="10" t="inlineStr">
         <is>
-          <t>Aperçu du corps JSON (POST /billing_subscriptions)</t>
+          <t>vat_rate</t>
+        </is>
+      </c>
+      <c r="N1" s="10" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="O1" s="10" t="inlineStr">
+        <is>
+          <t>payment_conditions</t>
+        </is>
+      </c>
+      <c r="P1" s="10" t="inlineStr">
+        <is>
+          <t>payment_method</t>
+        </is>
+      </c>
+      <c r="Q1" s="10" t="inlineStr">
+        <is>
+          <t>start (1er du mois suivant)</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="inlineStr">
+        <is>
+          <t>subscription_id existant</t>
+        </is>
+      </c>
+      <c r="S1" s="10" t="inlineStr">
+        <is>
+          <t>Corps JSON – POST /api/external/v2/billing_subscriptions</t>
         </is>
       </c>
     </row>
@@ -10519,7 +10609,7 @@
         <v/>
       </c>
       <c r="E2" s="15">
-        <f>"Loyer "&amp;INDEX(Baux!$B:$B,MATCH($A2,Baux!$A:$A,0))&amp;" – échéance "&amp;LOWER(F2)</f>
+        <f>"Loyer "&amp;INDEX(Baux!$B:$B,MATCH($A2,Baux!$A:$A,0))</f>
         <v/>
       </c>
       <c r="F2" s="15">
@@ -10527,31 +10617,55 @@
         <v/>
       </c>
       <c r="G2" s="15">
-        <f>IF(F2="Mensuelle","monthly",IF(F2="Trimestrielle","quarterly",IF(F2="Semestrielle","semiannual","yearly")))</f>
-        <v/>
-      </c>
-      <c r="H2" s="20">
+        <f>IF(F2="Annuelle","yearly","monthly")</f>
+        <v/>
+      </c>
+      <c r="H2" s="15">
+        <f>IF(F2="Mensuelle",1,IF(F2="Trimestrielle",3,IF(F2="Semestrielle",6,1)))</f>
+        <v/>
+      </c>
+      <c r="I2" s="15">
+        <f>IF(F2="Mensuelle","mois",IF(F2="Trimestrielle","trimestre",IF(F2="Semestrielle","semestre","an")))</f>
+        <v/>
+      </c>
+      <c r="J2" s="20">
         <f>ROUND(INDEX(Alertes!$G:$G,MATCH(A2,Alertes!$A:$A,0))/IF(F2="Mensuelle",12,IF(F2="Trimestrielle",4,IF(F2="Semestrielle",2,1))),2)</f>
         <v/>
       </c>
-      <c r="I2" s="20">
+      <c r="K2" s="20">
         <f>ROUND(IF(INDEX(Baux!$J:$J,MATCH($A2,Baux!$A:$A,0))="",0,INDEX(Baux!$J:$J,MATCH($A2,Baux!$A:$A,0)))/IF(F2="Mensuelle",12,IF(F2="Trimestrielle",4,IF(F2="Semestrielle",2,1))),2)</f>
         <v/>
       </c>
-      <c r="J2" s="15">
+      <c r="L2" s="15">
         <f>INDEX(Baux!$K:$K,MATCH($A2,Baux!$A:$A,0))</f>
         <v/>
       </c>
-      <c r="K2" s="15">
-        <f>IF(J2=20,"FR_200",IF(J2=10,"FR_100",IF(J2=5.5,"FR_55",IF(J2=2.1,"FR_21","exempt"))))</f>
-        <v/>
-      </c>
-      <c r="L2" s="13">
+      <c r="M2" s="15">
+        <f>IF(L2=20,"FR_200",IF(L2=10,"FR_100",IF(L2=5.5,"FR_55",IF(L2=2.1,"FR_21","exempt"))))</f>
+        <v/>
+      </c>
+      <c r="N2" s="15">
+        <f>Société!$B$11</f>
+        <v/>
+      </c>
+      <c r="O2" s="15">
+        <f>Société!$B$12</f>
+        <v/>
+      </c>
+      <c r="P2" s="15">
+        <f>Société!$B$13</f>
+        <v/>
+      </c>
+      <c r="Q2" s="13">
         <f>DATE(YEAR(TODAY()),MONTH(TODAY())+1,1)</f>
         <v/>
       </c>
-      <c r="M2" s="24">
-        <f>"{""customer_id"": "&amp;C2&amp;", ""start"": """&amp;YEAR(L2)&amp;"-"&amp;TEXT(MONTH(L2),"00")&amp;"-"&amp;TEXT(DAY(L2),"00")&amp;""", ""currency"": ""EUR"", ""recurrence"": {""type"": """&amp;G2&amp;""", ""day_of_month"": 1}, ""invoice_lines"": [{""label"": """&amp;E2&amp;""", ""quantity"": 1, ""raw_currency_unit_price"": "&amp;SUBSTITUTE(TEXT(H2,"0.00"),",",".")&amp;", ""vat_rate"": """&amp;K2&amp;""""&amp;IF(D2&lt;&gt;"",", ""product_id"": "&amp;D2,"")&amp;"}"&amp;IF(I2&gt;0,", {""label"": ""Provision sur charges"", ""quantity"": 1, ""raw_currency_unit_price"": "&amp;SUBSTITUTE(TEXT(I2,"0.00"),",",".")&amp;", ""vat_rate"": """&amp;K2&amp;"""}","")&amp;"]}"</f>
+      <c r="R2" s="15">
+        <f>IF(INDEX(Baux!$T:$T,MATCH($A2,Baux!$A:$A,0))="","",INDEX(Baux!$T:$T,MATCH($A2,Baux!$A:$A,0)))</f>
+        <v/>
+      </c>
+      <c r="S2" s="15">
+        <f>"{""customer_id"": "&amp;C2&amp;", ""label"": """&amp;E2&amp;""", ""start"": """&amp;YEAR(Q2)&amp;"-"&amp;TEXT(MONTH(Q2),"00")&amp;"-"&amp;TEXT(DAY(Q2),"00")&amp;""", ""mode"": {""type"": """&amp;N2&amp;"""}, ""payment_conditions"": """&amp;O2&amp;""", ""payment_method"": """&amp;P2&amp;""", ""recurring_rule"": "&amp;"{""type"": """&amp;G2&amp;""", ""interval"": "&amp;H2&amp;IF(G2="monthly",", ""day_of_month"": 1","")&amp;"}"&amp;", ""customer_invoice_data"": {""currency"": ""EUR"", ""language"": ""fr_FR"", ""pdf_invoice_subject"": """&amp;E2&amp;""", ""invoice_lines"": ["&amp;"{""label"": ""Loyer "&amp;LOWER(F2)&amp;" – "&amp;INDEX(Baux!$B:$B,MATCH($A2,Baux!$A:$A,0))&amp;""", ""quantity"": 1, ""unit"": """&amp;I2&amp;""", ""raw_currency_unit_price"": """&amp;SUBSTITUTE(TEXT(J2,"0.00"),",",".")&amp;""", ""vat_rate"": """&amp;M2&amp;""""&amp;IF(D2&lt;&gt;"",", ""product_id"": "&amp;D2,"")&amp;"}"&amp;IF(K2&gt;0,", {""label"": ""Provision sur charges"", ""quantity"": 1, ""unit"": """&amp;I2&amp;""", ""raw_currency_unit_price"": """&amp;SUBSTITUTE(TEXT(K2,"0.00"),",",".")&amp;""", ""vat_rate"": """&amp;M2&amp;"""}","")&amp;"]}}"</f>
         <v/>
       </c>
     </row>
@@ -10574,7 +10688,7 @@
         <v/>
       </c>
       <c r="E3" s="15">
-        <f>"Loyer "&amp;INDEX(Baux!$B:$B,MATCH($A3,Baux!$A:$A,0))&amp;" – échéance "&amp;LOWER(F3)</f>
+        <f>"Loyer "&amp;INDEX(Baux!$B:$B,MATCH($A3,Baux!$A:$A,0))</f>
         <v/>
       </c>
       <c r="F3" s="15">
@@ -10582,31 +10696,55 @@
         <v/>
       </c>
       <c r="G3" s="15">
-        <f>IF(F3="Mensuelle","monthly",IF(F3="Trimestrielle","quarterly",IF(F3="Semestrielle","semiannual","yearly")))</f>
-        <v/>
-      </c>
-      <c r="H3" s="20">
+        <f>IF(F3="Annuelle","yearly","monthly")</f>
+        <v/>
+      </c>
+      <c r="H3" s="15">
+        <f>IF(F3="Mensuelle",1,IF(F3="Trimestrielle",3,IF(F3="Semestrielle",6,1)))</f>
+        <v/>
+      </c>
+      <c r="I3" s="15">
+        <f>IF(F3="Mensuelle","mois",IF(F3="Trimestrielle","trimestre",IF(F3="Semestrielle","semestre","an")))</f>
+        <v/>
+      </c>
+      <c r="J3" s="20">
         <f>ROUND(INDEX(Alertes!$G:$G,MATCH(A3,Alertes!$A:$A,0))/IF(F3="Mensuelle",12,IF(F3="Trimestrielle",4,IF(F3="Semestrielle",2,1))),2)</f>
         <v/>
       </c>
-      <c r="I3" s="20">
+      <c r="K3" s="20">
         <f>ROUND(IF(INDEX(Baux!$J:$J,MATCH($A3,Baux!$A:$A,0))="",0,INDEX(Baux!$J:$J,MATCH($A3,Baux!$A:$A,0)))/IF(F3="Mensuelle",12,IF(F3="Trimestrielle",4,IF(F3="Semestrielle",2,1))),2)</f>
         <v/>
       </c>
-      <c r="J3" s="15">
+      <c r="L3" s="15">
         <f>INDEX(Baux!$K:$K,MATCH($A3,Baux!$A:$A,0))</f>
         <v/>
       </c>
-      <c r="K3" s="15">
-        <f>IF(J3=20,"FR_200",IF(J3=10,"FR_100",IF(J3=5.5,"FR_55",IF(J3=2.1,"FR_21","exempt"))))</f>
-        <v/>
-      </c>
-      <c r="L3" s="13">
+      <c r="M3" s="15">
+        <f>IF(L3=20,"FR_200",IF(L3=10,"FR_100",IF(L3=5.5,"FR_55",IF(L3=2.1,"FR_21","exempt"))))</f>
+        <v/>
+      </c>
+      <c r="N3" s="15">
+        <f>Société!$B$11</f>
+        <v/>
+      </c>
+      <c r="O3" s="15">
+        <f>Société!$B$12</f>
+        <v/>
+      </c>
+      <c r="P3" s="15">
+        <f>Société!$B$13</f>
+        <v/>
+      </c>
+      <c r="Q3" s="13">
         <f>DATE(YEAR(TODAY()),MONTH(TODAY())+1,1)</f>
         <v/>
       </c>
-      <c r="M3" s="24">
-        <f>"{""customer_id"": "&amp;C3&amp;", ""start"": """&amp;YEAR(L3)&amp;"-"&amp;TEXT(MONTH(L3),"00")&amp;"-"&amp;TEXT(DAY(L3),"00")&amp;""", ""currency"": ""EUR"", ""recurrence"": {""type"": """&amp;G3&amp;""", ""day_of_month"": 1}, ""invoice_lines"": [{""label"": """&amp;E3&amp;""", ""quantity"": 1, ""raw_currency_unit_price"": "&amp;SUBSTITUTE(TEXT(H3,"0.00"),",",".")&amp;", ""vat_rate"": """&amp;K3&amp;""""&amp;IF(D3&lt;&gt;"",", ""product_id"": "&amp;D3,"")&amp;"}"&amp;IF(I3&gt;0,", {""label"": ""Provision sur charges"", ""quantity"": 1, ""raw_currency_unit_price"": "&amp;SUBSTITUTE(TEXT(I3,"0.00"),",",".")&amp;", ""vat_rate"": """&amp;K3&amp;"""}","")&amp;"]}"</f>
+      <c r="R3" s="15">
+        <f>IF(INDEX(Baux!$T:$T,MATCH($A3,Baux!$A:$A,0))="","",INDEX(Baux!$T:$T,MATCH($A3,Baux!$A:$A,0)))</f>
+        <v/>
+      </c>
+      <c r="S3" s="15">
+        <f>"{""customer_id"": "&amp;C3&amp;", ""label"": """&amp;E3&amp;""", ""start"": """&amp;YEAR(Q3)&amp;"-"&amp;TEXT(MONTH(Q3),"00")&amp;"-"&amp;TEXT(DAY(Q3),"00")&amp;""", ""mode"": {""type"": """&amp;N3&amp;"""}, ""payment_conditions"": """&amp;O3&amp;""", ""payment_method"": """&amp;P3&amp;""", ""recurring_rule"": "&amp;"{""type"": """&amp;G3&amp;""", ""interval"": "&amp;H3&amp;IF(G3="monthly",", ""day_of_month"": 1","")&amp;"}"&amp;", ""customer_invoice_data"": {""currency"": ""EUR"", ""language"": ""fr_FR"", ""pdf_invoice_subject"": """&amp;E3&amp;""", ""invoice_lines"": ["&amp;"{""label"": ""Loyer "&amp;LOWER(F3)&amp;" – "&amp;INDEX(Baux!$B:$B,MATCH($A3,Baux!$A:$A,0))&amp;""", ""quantity"": 1, ""unit"": """&amp;I3&amp;""", ""raw_currency_unit_price"": """&amp;SUBSTITUTE(TEXT(J3,"0.00"),",",".")&amp;""", ""vat_rate"": """&amp;M3&amp;""""&amp;IF(D3&lt;&gt;"",", ""product_id"": "&amp;D3,"")&amp;"}"&amp;IF(K3&gt;0,", {""label"": ""Provision sur charges"", ""quantity"": 1, ""unit"": """&amp;I3&amp;""", ""raw_currency_unit_price"": """&amp;SUBSTITUTE(TEXT(K3,"0.00"),",",".")&amp;""", ""vat_rate"": """&amp;M3&amp;"""}","")&amp;"]}}"</f>
         <v/>
       </c>
     </row>
@@ -10629,7 +10767,7 @@
         <v/>
       </c>
       <c r="E4" s="15">
-        <f>"Loyer "&amp;INDEX(Baux!$B:$B,MATCH($A4,Baux!$A:$A,0))&amp;" – échéance "&amp;LOWER(F4)</f>
+        <f>"Loyer "&amp;INDEX(Baux!$B:$B,MATCH($A4,Baux!$A:$A,0))</f>
         <v/>
       </c>
       <c r="F4" s="15">
@@ -10637,31 +10775,55 @@
         <v/>
       </c>
       <c r="G4" s="15">
-        <f>IF(F4="Mensuelle","monthly",IF(F4="Trimestrielle","quarterly",IF(F4="Semestrielle","semiannual","yearly")))</f>
-        <v/>
-      </c>
-      <c r="H4" s="20">
+        <f>IF(F4="Annuelle","yearly","monthly")</f>
+        <v/>
+      </c>
+      <c r="H4" s="15">
+        <f>IF(F4="Mensuelle",1,IF(F4="Trimestrielle",3,IF(F4="Semestrielle",6,1)))</f>
+        <v/>
+      </c>
+      <c r="I4" s="15">
+        <f>IF(F4="Mensuelle","mois",IF(F4="Trimestrielle","trimestre",IF(F4="Semestrielle","semestre","an")))</f>
+        <v/>
+      </c>
+      <c r="J4" s="20">
         <f>ROUND(INDEX(Alertes!$G:$G,MATCH(A4,Alertes!$A:$A,0))/IF(F4="Mensuelle",12,IF(F4="Trimestrielle",4,IF(F4="Semestrielle",2,1))),2)</f>
         <v/>
       </c>
-      <c r="I4" s="20">
+      <c r="K4" s="20">
         <f>ROUND(IF(INDEX(Baux!$J:$J,MATCH($A4,Baux!$A:$A,0))="",0,INDEX(Baux!$J:$J,MATCH($A4,Baux!$A:$A,0)))/IF(F4="Mensuelle",12,IF(F4="Trimestrielle",4,IF(F4="Semestrielle",2,1))),2)</f>
         <v/>
       </c>
-      <c r="J4" s="15">
+      <c r="L4" s="15">
         <f>INDEX(Baux!$K:$K,MATCH($A4,Baux!$A:$A,0))</f>
         <v/>
       </c>
-      <c r="K4" s="15">
-        <f>IF(J4=20,"FR_200",IF(J4=10,"FR_100",IF(J4=5.5,"FR_55",IF(J4=2.1,"FR_21","exempt"))))</f>
-        <v/>
-      </c>
-      <c r="L4" s="13">
+      <c r="M4" s="15">
+        <f>IF(L4=20,"FR_200",IF(L4=10,"FR_100",IF(L4=5.5,"FR_55",IF(L4=2.1,"FR_21","exempt"))))</f>
+        <v/>
+      </c>
+      <c r="N4" s="15">
+        <f>Société!$B$11</f>
+        <v/>
+      </c>
+      <c r="O4" s="15">
+        <f>Société!$B$12</f>
+        <v/>
+      </c>
+      <c r="P4" s="15">
+        <f>Société!$B$13</f>
+        <v/>
+      </c>
+      <c r="Q4" s="13">
         <f>DATE(YEAR(TODAY()),MONTH(TODAY())+1,1)</f>
         <v/>
       </c>
-      <c r="M4" s="24">
-        <f>"{""customer_id"": "&amp;C4&amp;", ""start"": """&amp;YEAR(L4)&amp;"-"&amp;TEXT(MONTH(L4),"00")&amp;"-"&amp;TEXT(DAY(L4),"00")&amp;""", ""currency"": ""EUR"", ""recurrence"": {""type"": """&amp;G4&amp;""", ""day_of_month"": 1}, ""invoice_lines"": [{""label"": """&amp;E4&amp;""", ""quantity"": 1, ""raw_currency_unit_price"": "&amp;SUBSTITUTE(TEXT(H4,"0.00"),",",".")&amp;", ""vat_rate"": """&amp;K4&amp;""""&amp;IF(D4&lt;&gt;"",", ""product_id"": "&amp;D4,"")&amp;"}"&amp;IF(I4&gt;0,", {""label"": ""Provision sur charges"", ""quantity"": 1, ""raw_currency_unit_price"": "&amp;SUBSTITUTE(TEXT(I4,"0.00"),",",".")&amp;", ""vat_rate"": """&amp;K4&amp;"""}","")&amp;"]}"</f>
+      <c r="R4" s="15">
+        <f>IF(INDEX(Baux!$T:$T,MATCH($A4,Baux!$A:$A,0))="","",INDEX(Baux!$T:$T,MATCH($A4,Baux!$A:$A,0)))</f>
+        <v/>
+      </c>
+      <c r="S4" s="15">
+        <f>"{""customer_id"": "&amp;C4&amp;", ""label"": """&amp;E4&amp;""", ""start"": """&amp;YEAR(Q4)&amp;"-"&amp;TEXT(MONTH(Q4),"00")&amp;"-"&amp;TEXT(DAY(Q4),"00")&amp;""", ""mode"": {""type"": """&amp;N4&amp;"""}, ""payment_conditions"": """&amp;O4&amp;""", ""payment_method"": """&amp;P4&amp;""", ""recurring_rule"": "&amp;"{""type"": """&amp;G4&amp;""", ""interval"": "&amp;H4&amp;IF(G4="monthly",", ""day_of_month"": 1","")&amp;"}"&amp;", ""customer_invoice_data"": {""currency"": ""EUR"", ""language"": ""fr_FR"", ""pdf_invoice_subject"": """&amp;E4&amp;""", ""invoice_lines"": ["&amp;"{""label"": ""Loyer "&amp;LOWER(F4)&amp;" – "&amp;INDEX(Baux!$B:$B,MATCH($A4,Baux!$A:$A,0))&amp;""", ""quantity"": 1, ""unit"": """&amp;I4&amp;""", ""raw_currency_unit_price"": """&amp;SUBSTITUTE(TEXT(J4,"0.00"),",",".")&amp;""", ""vat_rate"": """&amp;M4&amp;""""&amp;IF(D4&lt;&gt;"",", ""product_id"": "&amp;D4,"")&amp;"}"&amp;IF(K4&gt;0,", {""label"": ""Provision sur charges"", ""quantity"": 1, ""unit"": """&amp;I4&amp;""", ""raw_currency_unit_price"": """&amp;SUBSTITUTE(TEXT(K4,"0.00"),",",".")&amp;""", ""vat_rate"": """&amp;M4&amp;"""}","")&amp;"]}}"</f>
         <v/>
       </c>
     </row>
@@ -10684,7 +10846,7 @@
         <v/>
       </c>
       <c r="E5" s="15">
-        <f>"Loyer "&amp;INDEX(Baux!$B:$B,MATCH($A5,Baux!$A:$A,0))&amp;" – échéance "&amp;LOWER(F5)</f>
+        <f>"Loyer "&amp;INDEX(Baux!$B:$B,MATCH($A5,Baux!$A:$A,0))</f>
         <v/>
       </c>
       <c r="F5" s="15">
@@ -10692,38 +10854,62 @@
         <v/>
       </c>
       <c r="G5" s="15">
-        <f>IF(F5="Mensuelle","monthly",IF(F5="Trimestrielle","quarterly",IF(F5="Semestrielle","semiannual","yearly")))</f>
-        <v/>
-      </c>
-      <c r="H5" s="20">
+        <f>IF(F5="Annuelle","yearly","monthly")</f>
+        <v/>
+      </c>
+      <c r="H5" s="15">
+        <f>IF(F5="Mensuelle",1,IF(F5="Trimestrielle",3,IF(F5="Semestrielle",6,1)))</f>
+        <v/>
+      </c>
+      <c r="I5" s="15">
+        <f>IF(F5="Mensuelle","mois",IF(F5="Trimestrielle","trimestre",IF(F5="Semestrielle","semestre","an")))</f>
+        <v/>
+      </c>
+      <c r="J5" s="20">
         <f>ROUND(INDEX(Alertes!$G:$G,MATCH(A5,Alertes!$A:$A,0))/IF(F5="Mensuelle",12,IF(F5="Trimestrielle",4,IF(F5="Semestrielle",2,1))),2)</f>
         <v/>
       </c>
-      <c r="I5" s="20">
+      <c r="K5" s="20">
         <f>ROUND(IF(INDEX(Baux!$J:$J,MATCH($A5,Baux!$A:$A,0))="",0,INDEX(Baux!$J:$J,MATCH($A5,Baux!$A:$A,0)))/IF(F5="Mensuelle",12,IF(F5="Trimestrielle",4,IF(F5="Semestrielle",2,1))),2)</f>
         <v/>
       </c>
-      <c r="J5" s="15">
+      <c r="L5" s="15">
         <f>INDEX(Baux!$K:$K,MATCH($A5,Baux!$A:$A,0))</f>
         <v/>
       </c>
-      <c r="K5" s="15">
-        <f>IF(J5=20,"FR_200",IF(J5=10,"FR_100",IF(J5=5.5,"FR_55",IF(J5=2.1,"FR_21","exempt"))))</f>
-        <v/>
-      </c>
-      <c r="L5" s="13">
+      <c r="M5" s="15">
+        <f>IF(L5=20,"FR_200",IF(L5=10,"FR_100",IF(L5=5.5,"FR_55",IF(L5=2.1,"FR_21","exempt"))))</f>
+        <v/>
+      </c>
+      <c r="N5" s="15">
+        <f>Société!$B$11</f>
+        <v/>
+      </c>
+      <c r="O5" s="15">
+        <f>Société!$B$12</f>
+        <v/>
+      </c>
+      <c r="P5" s="15">
+        <f>Société!$B$13</f>
+        <v/>
+      </c>
+      <c r="Q5" s="13">
         <f>DATE(YEAR(TODAY()),MONTH(TODAY())+1,1)</f>
         <v/>
       </c>
-      <c r="M5" s="24">
-        <f>"{""customer_id"": "&amp;C5&amp;", ""start"": """&amp;YEAR(L5)&amp;"-"&amp;TEXT(MONTH(L5),"00")&amp;"-"&amp;TEXT(DAY(L5),"00")&amp;""", ""currency"": ""EUR"", ""recurrence"": {""type"": """&amp;G5&amp;""", ""day_of_month"": 1}, ""invoice_lines"": [{""label"": """&amp;E5&amp;""", ""quantity"": 1, ""raw_currency_unit_price"": "&amp;SUBSTITUTE(TEXT(H5,"0.00"),",",".")&amp;", ""vat_rate"": """&amp;K5&amp;""""&amp;IF(D5&lt;&gt;"",", ""product_id"": "&amp;D5,"")&amp;"}"&amp;IF(I5&gt;0,", {""label"": ""Provision sur charges"", ""quantity"": 1, ""raw_currency_unit_price"": "&amp;SUBSTITUTE(TEXT(I5,"0.00"),",",".")&amp;", ""vat_rate"": """&amp;K5&amp;"""}","")&amp;"]}"</f>
+      <c r="R5" s="15">
+        <f>IF(INDEX(Baux!$T:$T,MATCH($A5,Baux!$A:$A,0))="","",INDEX(Baux!$T:$T,MATCH($A5,Baux!$A:$A,0)))</f>
+        <v/>
+      </c>
+      <c r="S5" s="15">
+        <f>"{""customer_id"": "&amp;C5&amp;", ""label"": """&amp;E5&amp;""", ""start"": """&amp;YEAR(Q5)&amp;"-"&amp;TEXT(MONTH(Q5),"00")&amp;"-"&amp;TEXT(DAY(Q5),"00")&amp;""", ""mode"": {""type"": """&amp;N5&amp;"""}, ""payment_conditions"": """&amp;O5&amp;""", ""payment_method"": """&amp;P5&amp;""", ""recurring_rule"": "&amp;"{""type"": """&amp;G5&amp;""", ""interval"": "&amp;H5&amp;IF(G5="monthly",", ""day_of_month"": 1","")&amp;"}"&amp;", ""customer_invoice_data"": {""currency"": ""EUR"", ""language"": ""fr_FR"", ""pdf_invoice_subject"": """&amp;E5&amp;""", ""invoice_lines"": ["&amp;"{""label"": ""Loyer "&amp;LOWER(F5)&amp;" – "&amp;INDEX(Baux!$B:$B,MATCH($A5,Baux!$A:$A,0))&amp;""", ""quantity"": 1, ""unit"": """&amp;I5&amp;""", ""raw_currency_unit_price"": """&amp;SUBSTITUTE(TEXT(J5,"0.00"),",",".")&amp;""", ""vat_rate"": """&amp;M5&amp;""""&amp;IF(D5&lt;&gt;"",", ""product_id"": "&amp;D5,"")&amp;"}"&amp;IF(K5&gt;0,", {""label"": ""Provision sur charges"", ""quantity"": 1, ""unit"": """&amp;I5&amp;""", ""raw_currency_unit_price"": """&amp;SUBSTITUTE(TEXT(K5,"0.00"),",",".")&amp;""", ""vat_rate"": """&amp;M5&amp;"""}","")&amp;"]}}"</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Schéma indicatif : les noms de champs (recurrence, invoice_lines, raw_currency_unit_price, vat_rate) sont à valider contre https://pennylane.readme.io/reference/postbillingsubscriptions avant tout envoi. Le mapping est modifiable dans config/pennylane_mapping.json.</t>
+          <t>Schéma : OpenAPI Pennylane Company V2 (POST /billing_subscriptions, mise à jour 2026-05-27). Mode, conditions et moyen de paiement se règlent dans la feuille Société. L'envoi se fait par la commande pennylane &lt;société&gt; --push ; l'identifiant créé est inscrit dans Baux (Pennylane subscription_id).</t>
         </is>
       </c>
     </row>

</xml_diff>